<commit_message>
Mixer cost: printed top instead of aluminium plate + shelf (~$626)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CXWjNkDcKCLLMLmWGq6ToQ
</commit_message>
<xml_diff>
--- a/mixer/cost/mixer_cost.xlsx
+++ b/mixer/cost/mixer_cost.xlsx
@@ -483,11 +483,11 @@
         </is>
       </c>
       <c r="B2" s="2">
-        <f>SUMIF(Cost!A2:A56,A2,Cost!F2:F56)</f>
+        <f>SUMIF(Cost!A2:A55,A2,Cost!F2:F55)</f>
         <v/>
       </c>
       <c r="C2" s="2">
-        <f>SUMIFS(Cost!F2:F56,Cost!A2:A56,A2,Cost!H2:H56,"estimate")</f>
+        <f>SUMIFS(Cost!F2:F55,Cost!A2:A55,A2,Cost!H2:H55,"estimate")</f>
         <v/>
       </c>
     </row>
@@ -498,11 +498,11 @@
         </is>
       </c>
       <c r="B3" s="2">
-        <f>SUMIF(Cost!A2:A56,A3,Cost!F2:F56)</f>
+        <f>SUMIF(Cost!A2:A55,A3,Cost!F2:F55)</f>
         <v/>
       </c>
       <c r="C3" s="2">
-        <f>SUMIFS(Cost!F2:F56,Cost!A2:A56,A3,Cost!H2:H56,"estimate")</f>
+        <f>SUMIFS(Cost!F2:F55,Cost!A2:A55,A3,Cost!H2:H55,"estimate")</f>
         <v/>
       </c>
     </row>
@@ -513,11 +513,11 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>SUMIF(Cost!A2:A56,A4,Cost!F2:F56)</f>
+        <f>SUMIF(Cost!A2:A55,A4,Cost!F2:F55)</f>
         <v/>
       </c>
       <c r="C4" s="2">
-        <f>SUMIFS(Cost!F2:F56,Cost!A2:A56,A4,Cost!H2:H56,"estimate")</f>
+        <f>SUMIFS(Cost!F2:F55,Cost!A2:A55,A4,Cost!H2:H55,"estimate")</f>
         <v/>
       </c>
     </row>
@@ -528,11 +528,11 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>SUMIF(Cost!A2:A56,A5,Cost!F2:F56)</f>
+        <f>SUMIF(Cost!A2:A55,A5,Cost!F2:F55)</f>
         <v/>
       </c>
       <c r="C5" s="2">
-        <f>SUMIFS(Cost!F2:F56,Cost!A2:A56,A5,Cost!H2:H56,"estimate")</f>
+        <f>SUMIFS(Cost!F2:F55,Cost!A2:A55,A5,Cost!H2:H55,"estimate")</f>
         <v/>
       </c>
     </row>
@@ -543,11 +543,11 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <f>SUMIF(Cost!A2:A56,A6,Cost!F2:F56)</f>
+        <f>SUMIF(Cost!A2:A55,A6,Cost!F2:F55)</f>
         <v/>
       </c>
       <c r="C6" s="2">
-        <f>SUMIFS(Cost!F2:F56,Cost!A2:A56,A6,Cost!H2:H56,"estimate")</f>
+        <f>SUMIFS(Cost!F2:F55,Cost!A2:A55,A6,Cost!H2:H55,"estimate")</f>
         <v/>
       </c>
     </row>
@@ -558,11 +558,11 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>SUMIF(Cost!A2:A56,A7,Cost!F2:F56)</f>
+        <f>SUMIF(Cost!A2:A55,A7,Cost!F2:F55)</f>
         <v/>
       </c>
       <c r="C7" s="2">
-        <f>SUMIFS(Cost!F2:F56,Cost!A2:A56,A7,Cost!H2:H56,"estimate")</f>
+        <f>SUMIFS(Cost!F2:F55,Cost!A2:A55,A7,Cost!H2:H55,"estimate")</f>
         <v/>
       </c>
     </row>
@@ -573,11 +573,11 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <f>SUMIF(Cost!A2:A56,A8,Cost!F2:F56)</f>
+        <f>SUMIF(Cost!A2:A55,A8,Cost!F2:F55)</f>
         <v/>
       </c>
       <c r="C8" s="2">
-        <f>SUMIFS(Cost!F2:F56,Cost!A2:A56,A8,Cost!H2:H56,"estimate")</f>
+        <f>SUMIFS(Cost!F2:F55,Cost!A2:A55,A8,Cost!H2:H55,"estimate")</f>
         <v/>
       </c>
     </row>
@@ -588,11 +588,11 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <f>SUMIF(Cost!A2:A56,A9,Cost!F2:F56)</f>
+        <f>SUMIF(Cost!A2:A55,A9,Cost!F2:F55)</f>
         <v/>
       </c>
       <c r="C9" s="2">
-        <f>SUMIFS(Cost!F2:F56,Cost!A2:A56,A9,Cost!H2:H56,"estimate")</f>
+        <f>SUMIFS(Cost!F2:F55,Cost!A2:A55,A9,Cost!H2:H55,"estimate")</f>
         <v/>
       </c>
     </row>
@@ -603,11 +603,11 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <f>SUMIF(Cost!A2:A56,A10,Cost!F2:F56)</f>
+        <f>SUMIF(Cost!A2:A55,A10,Cost!F2:F55)</f>
         <v/>
       </c>
       <c r="C10" s="2">
-        <f>SUMIFS(Cost!F2:F56,Cost!A2:A56,A10,Cost!H2:H56,"estimate")</f>
+        <f>SUMIFS(Cost!F2:F55,Cost!A2:A55,A10,Cost!H2:H55,"estimate")</f>
         <v/>
       </c>
     </row>
@@ -618,11 +618,11 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <f>SUMIF(Cost!A2:A56,A11,Cost!F2:F56)</f>
+        <f>SUMIF(Cost!A2:A55,A11,Cost!F2:F55)</f>
         <v/>
       </c>
       <c r="C11" s="2">
-        <f>SUMIFS(Cost!F2:F56,Cost!A2:A56,A11,Cost!H2:H56,"estimate")</f>
+        <f>SUMIFS(Cost!F2:F55,Cost!A2:A55,A11,Cost!H2:H55,"estimate")</f>
         <v/>
       </c>
     </row>
@@ -633,11 +633,11 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <f>SUMIF(Cost!A2:A56,A12,Cost!F2:F56)</f>
+        <f>SUMIF(Cost!A2:A55,A12,Cost!F2:F55)</f>
         <v/>
       </c>
       <c r="C12" s="2">
-        <f>SUMIFS(Cost!F2:F56,Cost!A2:A56,A12,Cost!H2:H56,"estimate")</f>
+        <f>SUMIFS(Cost!F2:F55,Cost!A2:A55,A12,Cost!H2:H55,"estimate")</f>
         <v/>
       </c>
     </row>
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2325,19 +2325,19 @@
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Control plate</t>
+          <t>Printed top (control plate + jack shelf)</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>407x292 mm, 2.0 mm 5052 aluminium, 141 cuts (plate.dxf)</t>
+          <t>Omer chose printed over aluminium 2026-10-27; PLA ~0.45 kg, split into bed-size tiles</t>
         </is>
       </c>
       <c r="D44" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E44" s="8" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="F44" s="8">
         <f>D44*E44</f>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>SendCutSend</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
@@ -2362,19 +2362,19 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Jack shelf</t>
+          <t>Filament</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>407x180 mm, 1.5 mm 5052 aluminium, 46 cuts (shelf.dxf)</t>
+          <t>PLA 2 spools: case ~0.8 kg + printed top ~0.45 kg + spare</t>
         </is>
       </c>
       <c r="D45" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E45" s="8" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="F45" s="8">
         <f>D45*E45</f>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>SendCutSend</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
@@ -2399,19 +2399,19 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Filament</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>PLA ~0.8 kg (923 cm3 solid STL volume at ~60% fill)</t>
+          <t>M3 F-F standoffs 10.5/7.5 mm, M3x10 countersunk, M2x8 + 4 mm spacers, seam bolts</t>
         </is>
       </c>
       <c r="D46" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E46" s="8" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F46" s="8">
         <f>D46*E46</f>
@@ -2429,76 +2429,76 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="inlineStr">
+      <c r="A47" s="9" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t>Hardware</t>
-        </is>
-      </c>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>M3 F-F standoffs 10.5/7.5 mm, M3x10 countersunk, M2x8 + 4 mm spacers, seam bolts</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E47" s="8" t="n">
-        <v>15</v>
-      </c>
-      <c r="F47" s="8">
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>M3 screws + heat-set inserts</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Already bought for the controller</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="10">
         <f>D47*E47</f>
         <v/>
       </c>
-      <c r="G47" s="7" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="H47" s="7" t="inlineStr">
-        <is>
-          <t>estimate</t>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="inlineStr">
+        <is>
+          <t>owned</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="9" t="inlineStr">
-        <is>
-          <t>Case</t>
-        </is>
-      </c>
-      <c r="B48" s="9" t="inlineStr">
-        <is>
-          <t>M3 screws + heat-set inserts</t>
-        </is>
-      </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>Already bought for the controller</t>
-        </is>
-      </c>
-      <c r="D48" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E48" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F48" s="10">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>Knobs</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Pot knobs</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>41 knobs, 6.35 mm round shaft</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="E48" s="8" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F48" s="8">
         <f>D48*E48</f>
         <v/>
       </c>
-      <c r="G48" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H48" s="9" t="inlineStr">
-        <is>
-          <t>owned</t>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>Tayda</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
         </is>
       </c>
     </row>
@@ -2510,19 +2510,19 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Pot knobs</t>
+          <t>Fader caps</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>41 knobs, 6.35 mm round shaft</t>
+          <t>7 caps for PTA 15 mm metal lever</t>
         </is>
       </c>
       <c r="D49" s="7" t="n">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="E49" s="8" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="F49" s="8">
         <f>D49*E49</f>
@@ -2530,7 +2530,7 @@
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>Tayda</t>
+          <t>AliExpress</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
@@ -2547,19 +2547,19 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Fader caps</t>
+          <t>Controller knobs</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>7 caps for PTA 15 mm metal lever</t>
+          <t>4 fader caps + 4 encoder knobs</t>
         </is>
       </c>
       <c r="D50" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E50" s="8" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F50" s="8">
         <f>D50*E50</f>
@@ -2577,100 +2577,100 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="inlineStr">
-        <is>
-          <t>Knobs</t>
-        </is>
-      </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>Controller knobs</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>4 fader caps + 4 encoder knobs</t>
-        </is>
-      </c>
-      <c r="D51" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E51" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F51" s="8">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>ESP32-S3 devkit, 2.8" TFT, 45 mm faders, EC11s, buttons, LEDs, resistors</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>Already bought</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="10">
         <f>D51*E51</f>
         <v/>
       </c>
-      <c r="G51" s="7" t="inlineStr">
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H51" s="9" t="inlineStr">
+        <is>
+          <t>owned</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Headers</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Female 2.54 mm strips</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F52" s="8">
+        <f>D52*E52</f>
+        <v/>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
         <is>
           <t>AliExpress</t>
         </is>
       </c>
-      <c r="H51" s="7" t="inlineStr">
-        <is>
-          <t>estimate</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="9" t="inlineStr">
-        <is>
-          <t>Controller</t>
-        </is>
-      </c>
-      <c r="B52" s="9" t="inlineStr">
-        <is>
-          <t>ESP32-S3 devkit, 2.8" TFT, 45 mm faders, EC11s, buttons, LEDs, resistors</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>Already bought</t>
-        </is>
-      </c>
-      <c r="D52" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E52" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F52" s="10">
-        <f>D52*E52</f>
-        <v/>
-      </c>
-      <c r="G52" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H52" s="9" t="inlineStr">
-        <is>
-          <t>owned</t>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>Controller</t>
+          <t>Shipping</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Headers</t>
+          <t>DigiKey / Mouser</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Female 2.54 mm strips</t>
+          <t>Free over the order threshold</t>
         </is>
       </c>
       <c r="D53" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E53" s="8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F53" s="8">
         <f>D53*E53</f>
@@ -2678,7 +2678,7 @@
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>DigiKey</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
@@ -2695,19 +2695,19 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>DigiKey / Mouser</t>
+          <t>Tayda</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Free over the order threshold</t>
+          <t>To US</t>
         </is>
       </c>
       <c r="D54" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E54" s="8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F54" s="8">
         <f>D54*E54</f>
@@ -2715,7 +2715,7 @@
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>Tayda</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr">
@@ -2732,19 +2732,19 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>Tayda</t>
+          <t>Jameco</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>To US</t>
+          <t>Ground</t>
         </is>
       </c>
       <c r="D55" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E55" s="8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F55" s="8">
         <f>D55*E55</f>
@@ -2752,47 +2752,10 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>Tayda</t>
+          <t>Jameco</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr">
-        <is>
-          <t>estimate</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t>Shipping</t>
-        </is>
-      </c>
-      <c r="B56" s="7" t="inlineStr">
-        <is>
-          <t>Jameco</t>
-        </is>
-      </c>
-      <c r="C56" s="7" t="inlineStr">
-        <is>
-          <t>Ground</t>
-        </is>
-      </c>
-      <c r="D56" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="8" t="n">
-        <v>9</v>
-      </c>
-      <c r="F56" s="8">
-        <f>D56*E56</f>
-        <v/>
-      </c>
-      <c r="G56" s="7" t="inlineStr">
-        <is>
-          <t>Jameco</t>
-        </is>
-      </c>
-      <c r="H56" s="7" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>

</xml_diff>

<commit_message>
Mixer cost: add JLCPCB-assembled option (~$1,186 vs ~$626 DIY)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CXWjNkDcKCLLMLmWGq6ToQ
</commit_message>
<xml_diff>
--- a/mixer/cost/mixer_cost.xlsx
+++ b/mixer/cost/mixer_cost.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assembled" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -72,7 +73,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -80,10 +81,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -708,6 +710,343 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Unit $</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Total $</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Where</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>DIY total (Cost sheet)</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Everything above, you solder it</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="6">
+        <f>SUM(Cost!F2:F55)</f>
+        <v/>
+      </c>
+      <c r="E2" s="6">
+        <f>C2*D2</f>
+        <v/>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Assembly labour</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3198 through-hole joints x $0.0164</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>3198</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>0.0164</v>
+      </c>
+      <c r="E3" s="7">
+        <f>C3*D3</f>
+        <v/>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Setup + stencil</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>7 designs x ($8.18 + $1.53)</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>9.710000000000001</v>
+      </c>
+      <c r="E4" s="7">
+        <f>C4*D4</f>
+        <v/>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hand-soldering fee</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>per order</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="E5" s="7">
+        <f>C5*D5</f>
+        <v/>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Parts for the 2-board minimum</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>2nd master, power, digital, reverb boards (~$68 master, rest smaller)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>105</v>
+      </c>
+      <c r="E6" s="6">
+        <f>C6*D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>JLC parts markup</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>~25% over DigiKey/Mouser on ~$330 of board parts (global sourcing for Neutrik, THAT, PTA, PVA2)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="E7" s="6">
+        <f>C7*D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>US import duty</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>~35% (Section 301 25% + 122 tariff 10%) on ~$640 of assembled boards</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>224</v>
+      </c>
+      <c r="E8" s="6">
+        <f>C8*D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>JLCPCB DDP</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Heavier DHL shipping</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>~2.5 kg of built boards vs ~1.5 kg bare</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="E9" s="6">
+        <f>C9*D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL, boards assembled</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>You still mount boards in the case, plug ribbons, fit the FV-1/hub/PCM2902 modules and knobs</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8">
+        <f>SUM(E2:E9)</f>
+        <v/>
+      </c>
+      <c r="F10" s="1" t="n"/>
+      <c r="G10" s="1" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -722,42 +1061,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Section</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>Part / note</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>Unit $</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>Total $</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>Where</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
@@ -782,10 +1121,10 @@
       <c r="D2" t="n">
         <v>4</v>
       </c>
-      <c r="E2" s="6" t="n">
+      <c r="E2" s="7" t="n">
         <v>5.84</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2" s="7">
         <f>D2*E2</f>
         <v/>
       </c>
@@ -801,148 +1140,148 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Chips</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Op-amps</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>NE5532P (12 strips + 4 master + 8 stereo)</t>
         </is>
       </c>
-      <c r="D3" s="7" t="n">
+      <c r="D3" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="6" t="n">
         <v>0.55</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="6">
         <f>D3*E3</f>
         <v/>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Tayda</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Chips</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Comparators</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>LM393 (4 strips + 4 stereo)</t>
         </is>
       </c>
-      <c r="D4" s="7" t="n">
+      <c r="D4" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="6" t="n">
         <v>0.35</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="6">
         <f>D4*E4</f>
         <v/>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Tayda</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Chips</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Peak op-amp</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>TL072CP (master)</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="8" t="n">
+      <c r="D5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="6" t="n">
         <v>0.6</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="6">
         <f>D5*E5</f>
         <v/>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Tayda</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Chips</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Balanced line drivers</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>TI DRV134PA (master)</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="6" t="n">
         <v>6.5</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="6">
         <f>D6*E6</f>
         <v/>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Mouser</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
@@ -967,10 +1306,10 @@
       <c r="D7" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="E7" s="7" t="n">
         <v>1.52</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="7">
         <f>D7*E7</f>
         <v/>
       </c>
@@ -986,111 +1325,111 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Chips</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Meter drivers</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>LM3915N-1 or NTE1509 (master)</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="6">
         <f>D8*E8</f>
         <v/>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Jameco / Mouser</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Chips</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>MIDI opto, reverb LDO + op-amp</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>6N138, MCP1700-3302E, MCP6002-I/P</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="8" t="n">
+      <c r="D9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="6">
         <f>D9*E9</f>
         <v/>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Chips</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>IC sockets</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>43x DIP-8 + 2x DIP-18</t>
         </is>
       </c>
-      <c r="D10" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="8" t="n">
+      <c r="D10" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="6" t="n">
         <v>3.5</v>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="6">
         <f>D10*E10</f>
         <v/>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Tayda</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
@@ -1115,10 +1454,10 @@
       <c r="D11" t="n">
         <v>4</v>
       </c>
-      <c r="E11" s="6" t="n">
+      <c r="E11" s="7" t="n">
         <v>2.37</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="7">
         <f>D11*E11</f>
         <v/>
       </c>
@@ -1134,37 +1473,37 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Controls</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Fader, dual (master + 2 stereo)</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Bourns PTA6044-2015DPA103 (DigiKey: 2000 MOQ, buy at Mouser/Utmel)</t>
         </is>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="6" t="n">
         <v>2.7</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="6">
         <f>D12*E12</f>
         <v/>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>Mouser / Utmel</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
@@ -1189,10 +1528,10 @@
       <c r="D13" t="n">
         <v>14</v>
       </c>
-      <c r="E13" s="6" t="n">
+      <c r="E13" s="7" t="n">
         <v>1.29</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="7">
         <f>D13*E13</f>
         <v/>
       </c>
@@ -1208,111 +1547,111 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Controls</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Pot C10K gain</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Alpha RD901F-40-15R1-C10K</t>
         </is>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E14" s="8" t="n">
+      <c r="E14" s="6" t="n">
         <v>1.29</v>
       </c>
-      <c r="F14" s="8">
+      <c r="F14" s="6">
         <f>D14*E14</f>
         <v/>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>Tayda</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Controls</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Pot B10K centre detent</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Alpha RD901F-40-15R1-B10K-0CD (Tayda A-8401)</t>
         </is>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="E15" s="8" t="n">
+      <c r="E15" s="6" t="n">
         <v>1.4</v>
       </c>
-      <c r="F15" s="8">
+      <c r="F15" s="6">
         <f>D15*E15</f>
         <v/>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>Tayda</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Controls</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Pot dual (phones A10K, stereo EQ B10K)</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Alpha RD902F (Tayda A-6980 / A-6433)</t>
         </is>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D16" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="E16" s="6" t="n">
         <v>2.2</v>
       </c>
-      <c r="F16" s="8">
+      <c r="F16" s="6">
         <f>D16*E16</f>
         <v/>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>Tayda</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
@@ -1337,10 +1676,10 @@
       <c r="D17" t="n">
         <v>13</v>
       </c>
-      <c r="E17" s="6" t="n">
+      <c r="E17" s="7" t="n">
         <v>2.424</v>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="7">
         <f>D17*E17</f>
         <v/>
       </c>
@@ -1356,185 +1695,185 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Controls</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Switch caps</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>C&amp;K PVA push caps</t>
         </is>
       </c>
-      <c r="D18" s="7" t="n">
+      <c r="D18" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="E18" s="8" t="n">
+      <c r="E18" s="6" t="n">
         <v>0.6</v>
       </c>
-      <c r="F18" s="8">
+      <c r="F18" s="6">
         <f>D18*E18</f>
         <v/>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Controls</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Reverb trimmers</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Bourns 3296W 10k x4, 20k x1</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D19" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E19" s="8" t="n">
+      <c r="E19" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="F19" s="8">
+      <c r="F19" s="6">
         <f>D19*E19</f>
         <v/>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Connectors</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Mic combo jacks</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Neutrik NCJ6FA-V</t>
         </is>
       </c>
-      <c r="D20" s="7" t="n">
+      <c r="D20" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E20" s="8" t="n">
+      <c r="E20" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="F20" s="8">
+      <c r="F20" s="6">
         <f>D20*E20</f>
         <v/>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Connectors</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Main XLR out</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Neutrik NC3MAAV</t>
         </is>
       </c>
-      <c r="D21" s="7" t="n">
+      <c r="D21" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E21" s="8" t="n">
+      <c r="E21" s="6" t="n">
         <v>3.5</v>
       </c>
-      <c r="F21" s="8">
+      <c r="F21" s="6">
         <f>D21*E21</f>
         <v/>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Connectors</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>1/4" jacks, master</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Neutrik NJ3FD-V</t>
         </is>
       </c>
-      <c r="D22" s="7" t="n">
+      <c r="D22" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E22" s="8" t="n">
+      <c r="E22" s="6" t="n">
         <v>1.8</v>
       </c>
-      <c r="F22" s="8">
+      <c r="F22" s="6">
         <f>D22*E22</f>
         <v/>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
@@ -1559,10 +1898,10 @@
       <c r="D23" t="n">
         <v>2</v>
       </c>
-      <c r="E23" s="6" t="n">
+      <c r="E23" s="7" t="n">
         <v>1.63</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="7">
         <f>D23*E23</f>
         <v/>
       </c>
@@ -1578,296 +1917,296 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Connectors</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>3.5 mm jacks</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Thonkiconn PJ366ST (master + stereo line)</t>
         </is>
       </c>
-      <c r="D24" s="7" t="n">
+      <c r="D24" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E24" s="8" t="n">
+      <c r="E24" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="F24" s="8">
+      <c r="F24" s="6">
         <f>D24*E24</f>
         <v/>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>Thonk</t>
         </is>
       </c>
-      <c r="H24" s="7" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Connectors</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>Shrouded 2x5 headers</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Wurth 61201021621</t>
         </is>
       </c>
-      <c r="D25" s="7" t="n">
+      <c r="D25" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="E25" s="8" t="n">
+      <c r="E25" s="6" t="n">
         <v>0.45</v>
       </c>
-      <c r="F25" s="8">
+      <c r="F25" s="6">
         <f>D25*E25</f>
         <v/>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>Mouser</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Connectors</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Ribbon cable + IDC plugs</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>2x5 IDC sockets x17 + 1 m 10-way ribbon</t>
         </is>
       </c>
-      <c r="D26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="8" t="n">
+      <c r="D26" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="F26" s="8">
+      <c r="F26" s="6">
         <f>D26*E26</f>
         <v/>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>Tayda</t>
         </is>
       </c>
-      <c r="H26" s="7" t="inlineStr">
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Connectors</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>Digital board jacks</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>USB-B, USB-C (GCT), USB-A, 2x DIN-5</t>
         </is>
       </c>
-      <c r="D27" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="8" t="n">
+      <c r="D27" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="F27" s="8">
+      <c r="F27" s="6">
         <f>D27*E27</f>
         <v/>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="H27" s="7" t="inlineStr">
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>Connectors</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Rear DC jack + pigtail</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Panel 2.1 mm jack, short 2.1 mm plug lead</t>
         </is>
       </c>
-      <c r="D28" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="8" t="n">
+      <c r="D28" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F28" s="8">
+      <c r="F28" s="6">
         <f>D28*E28</f>
         <v/>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>AliExpress</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Passives</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>Resistors</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>~320 metal film incl. 8x 0.1% 6.81k</t>
         </is>
       </c>
-      <c r="D29" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="8" t="n">
+      <c r="D29" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="F29" s="8">
+      <c r="F29" s="6">
         <f>D29*E29</f>
         <v/>
       </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="G29" s="5" t="inlineStr">
         <is>
           <t>Tayda</t>
         </is>
       </c>
-      <c r="H29" s="7" t="inlineStr">
+      <c r="H29" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Passives</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>Capacitors</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Films, ceramics, 7 mm low-profile electrolytics</t>
         </is>
       </c>
-      <c r="D30" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="8" t="n">
+      <c r="D30" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="F30" s="8">
+      <c r="F30" s="6">
         <f>D30*E30</f>
         <v/>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>Tayda / DigiKey</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Passives</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>LEDs, diodes, DIP switch, headers</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>3 mm LEDs, 1N4004/4148/5817, pin headers</t>
         </is>
       </c>
-      <c r="D31" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="8" t="n">
+      <c r="D31" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="F31" s="8">
+      <c r="F31" s="6">
         <f>D31*E31</f>
         <v/>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>Tayda</t>
         </is>
       </c>
-      <c r="H31" s="7" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
@@ -1892,10 +2231,10 @@
       <c r="D32" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="6" t="n">
+      <c r="E32" s="7" t="n">
         <v>10.95</v>
       </c>
-      <c r="F32" s="6">
+      <c r="F32" s="7">
         <f>D32*E32</f>
         <v/>
       </c>
@@ -1911,74 +2250,74 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>Power</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>Big caps</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>6800uF 35V snap-in x2, 1000uF 63V x4</t>
         </is>
       </c>
-      <c r="D33" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" s="8" t="n">
+      <c r="D33" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="F33" s="8">
+      <c r="F33" s="6">
         <f>D33*E33</f>
         <v/>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="H33" s="7" t="inlineStr">
+      <c r="H33" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="inlineStr">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>Power</t>
         </is>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>Regulators, heatsinks, fuse, rest</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>7812/7912, 2x Fischer SK104, MJE340, fuse + holder, barrel jack, insulator kit</t>
         </is>
       </c>
-      <c r="D34" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" s="8" t="n">
+      <c r="D34" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="F34" s="8">
+      <c r="F34" s="6">
         <f>D34*E34</f>
         <v/>
       </c>
-      <c r="G34" s="7" t="inlineStr">
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="H34" s="7" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
@@ -2003,10 +2342,10 @@
       <c r="D35" t="n">
         <v>1</v>
       </c>
-      <c r="E35" s="6" t="n">
+      <c r="E35" s="7" t="n">
         <v>18.5</v>
       </c>
-      <c r="F35" s="6">
+      <c r="F35" s="7">
         <f>D35*E35</f>
         <v/>
       </c>
@@ -2022,740 +2361,740 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="inlineStr">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>Modules</t>
         </is>
       </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>Proxy + Japan shipping</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>ZenMarket fee + EMS/small packet to US</t>
         </is>
       </c>
-      <c r="D36" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" s="8" t="n">
+      <c r="D36" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="F36" s="8">
+      <c r="F36" s="6">
         <f>D36*E36</f>
         <v/>
       </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="G36" s="5" t="inlineStr">
         <is>
           <t>ZenMarket</t>
         </is>
       </c>
-      <c r="H36" s="7" t="inlineStr">
+      <c r="H36" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="inlineStr">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Modules</t>
         </is>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>USB hub module</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>FE1.1s (Amazon JESSINIE)</t>
         </is>
       </c>
-      <c r="D37" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" s="8" t="n">
+      <c r="D37" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F37" s="8">
+      <c r="F37" s="6">
         <f>D37*E37</f>
         <v/>
       </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="H37" s="7" t="inlineStr">
+      <c r="H37" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>Modules</t>
         </is>
       </c>
-      <c r="B38" s="7" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>USB audio module</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>PCM2902 module</t>
         </is>
       </c>
-      <c r="D38" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="8" t="n">
+      <c r="D38" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F38" s="8">
+      <c r="F38" s="6">
         <f>D38*E38</f>
         <v/>
       </c>
-      <c r="G38" s="7" t="inlineStr">
+      <c r="G38" s="5" t="inlineStr">
         <is>
           <t>AliExpress</t>
         </is>
       </c>
-      <c r="H38" s="7" t="inlineStr">
+      <c r="H38" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="inlineStr">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>PCBs</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>Mono strip 30x343 mm</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>5 pcs (4 used)</t>
         </is>
       </c>
-      <c r="D39" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E39" s="8" t="n">
+      <c r="D39" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F39" s="8">
+      <c r="F39" s="6">
         <f>D39*E39</f>
         <v/>
       </c>
-      <c r="G39" s="7" t="inlineStr">
+      <c r="G39" s="5" t="inlineStr">
         <is>
           <t>JLCPCB</t>
         </is>
       </c>
-      <c r="H39" s="7" t="inlineStr">
+      <c r="H39" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="inlineStr">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>PCBs</t>
         </is>
       </c>
-      <c r="B40" s="7" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>Stereo strip 30x343 mm</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>5 pcs (2 used)</t>
         </is>
       </c>
-      <c r="D40" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E40" s="8" t="n">
+      <c r="D40" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F40" s="8">
+      <c r="F40" s="6">
         <f>D40*E40</f>
         <v/>
       </c>
-      <c r="G40" s="7" t="inlineStr">
+      <c r="G40" s="5" t="inlineStr">
         <is>
           <t>JLCPCB</t>
         </is>
       </c>
-      <c r="H40" s="7" t="inlineStr">
+      <c r="H40" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="inlineStr">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>PCBs</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>Master 60x343 mm</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>5 pcs (1 used)</t>
         </is>
       </c>
-      <c r="D41" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E41" s="8" t="n">
+      <c r="D41" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="F41" s="8">
+      <c r="F41" s="6">
         <f>D41*E41</f>
         <v/>
       </c>
-      <c r="G41" s="7" t="inlineStr">
+      <c r="G41" s="5" t="inlineStr">
         <is>
           <t>JLCPCB</t>
         </is>
       </c>
-      <c r="H41" s="7" t="inlineStr">
+      <c r="H41" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="inlineStr">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>PCBs</t>
         </is>
       </c>
-      <c r="B42" s="7" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>Power, digital, reverb, controller</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>4 small boards, 5 pcs each</t>
         </is>
       </c>
-      <c r="D42" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E42" s="8" t="n">
+      <c r="D42" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="F42" s="8">
+      <c r="F42" s="6">
         <f>D42*E42</f>
         <v/>
       </c>
-      <c r="G42" s="7" t="inlineStr">
+      <c r="G42" s="5" t="inlineStr">
         <is>
           <t>JLCPCB</t>
         </is>
       </c>
-      <c r="H42" s="7" t="inlineStr">
+      <c r="H42" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="inlineStr">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>PCBs</t>
         </is>
       </c>
-      <c r="B43" s="7" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>Shipping + import duty</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>DHL to US, ~1.5 kg</t>
         </is>
       </c>
-      <c r="D43" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E43" s="8" t="n">
+      <c r="D43" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="F43" s="8">
+      <c r="F43" s="6">
         <f>D43*E43</f>
         <v/>
       </c>
-      <c r="G43" s="7" t="inlineStr">
+      <c r="G43" s="5" t="inlineStr">
         <is>
           <t>JLCPCB</t>
         </is>
       </c>
-      <c r="H43" s="7" t="inlineStr">
+      <c r="H43" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="inlineStr">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="B44" s="7" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>Printed top (control plate + jack shelf)</t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>Omer chose printed over aluminium 2026-10-27; PLA ~0.45 kg, split into bed-size tiles</t>
         </is>
       </c>
-      <c r="D44" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" s="8" t="n">
+      <c r="D44" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F44" s="8">
+      <c r="F44" s="6">
         <f>D44*E44</f>
         <v/>
       </c>
-      <c r="G44" s="7" t="inlineStr">
+      <c r="G44" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H44" s="7" t="inlineStr">
+      <c r="H44" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>Filament</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>PLA 2 spools: case ~0.8 kg + printed top ~0.45 kg + spare</t>
         </is>
       </c>
-      <c r="D45" s="7" t="n">
+      <c r="D45" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E45" s="8" t="n">
+      <c r="E45" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="F45" s="8">
+      <c r="F45" s="6">
         <f>D45*E45</f>
         <v/>
       </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="G45" s="5" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="H45" s="7" t="inlineStr">
+      <c r="H45" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="inlineStr">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="B46" s="7" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="C46" s="7" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr">
         <is>
           <t>M3 F-F standoffs 10.5/7.5 mm, M3x10 countersunk, M2x8 + 4 mm spacers, seam bolts</t>
         </is>
       </c>
-      <c r="D46" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E46" s="8" t="n">
+      <c r="D46" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="F46" s="8">
+      <c r="F46" s="6">
         <f>D46*E46</f>
         <v/>
       </c>
-      <c r="G46" s="7" t="inlineStr">
+      <c r="G46" s="5" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="H46" s="7" t="inlineStr">
+      <c r="H46" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="9" t="inlineStr">
+      <c r="A47" s="10" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="B47" s="9" t="inlineStr">
+      <c r="B47" s="10" t="inlineStr">
         <is>
           <t>M3 screws + heat-set inserts</t>
         </is>
       </c>
-      <c r="C47" s="9" t="inlineStr">
+      <c r="C47" s="10" t="inlineStr">
         <is>
           <t>Already bought for the controller</t>
         </is>
       </c>
-      <c r="D47" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E47" s="10" t="n">
+      <c r="D47" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F47" s="10">
+      <c r="F47" s="11">
         <f>D47*E47</f>
         <v/>
       </c>
-      <c r="G47" s="9" t="inlineStr">
+      <c r="G47" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H47" s="9" t="inlineStr">
+      <c r="H47" s="10" t="inlineStr">
         <is>
           <t>owned</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="inlineStr">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>Knobs</t>
         </is>
       </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>Pot knobs</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr">
         <is>
           <t>41 knobs, 6.35 mm round shaft</t>
         </is>
       </c>
-      <c r="D48" s="7" t="n">
+      <c r="D48" s="5" t="n">
         <v>41</v>
       </c>
-      <c r="E48" s="8" t="n">
+      <c r="E48" s="6" t="n">
         <v>0.6</v>
       </c>
-      <c r="F48" s="8">
+      <c r="F48" s="6">
         <f>D48*E48</f>
         <v/>
       </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="G48" s="5" t="inlineStr">
         <is>
           <t>Tayda</t>
         </is>
       </c>
-      <c r="H48" s="7" t="inlineStr">
+      <c r="H48" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="inlineStr">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>Knobs</t>
         </is>
       </c>
-      <c r="B49" s="7" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>Fader caps</t>
         </is>
       </c>
-      <c r="C49" s="7" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>7 caps for PTA 15 mm metal lever</t>
         </is>
       </c>
-      <c r="D49" s="7" t="n">
+      <c r="D49" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="E49" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F49" s="8">
+      <c r="E49" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="6">
         <f>D49*E49</f>
         <v/>
       </c>
-      <c r="G49" s="7" t="inlineStr">
+      <c r="G49" s="5" t="inlineStr">
         <is>
           <t>AliExpress</t>
         </is>
       </c>
-      <c r="H49" s="7" t="inlineStr">
+      <c r="H49" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>Knobs</t>
         </is>
       </c>
-      <c r="B50" s="7" t="inlineStr">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>Controller knobs</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t>4 fader caps + 4 encoder knobs</t>
         </is>
       </c>
-      <c r="D50" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E50" s="8" t="n">
+      <c r="D50" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F50" s="8">
+      <c r="F50" s="6">
         <f>D50*E50</f>
         <v/>
       </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="G50" s="5" t="inlineStr">
         <is>
           <t>AliExpress</t>
         </is>
       </c>
-      <c r="H50" s="7" t="inlineStr">
+      <c r="H50" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="9" t="inlineStr">
+      <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Controller</t>
         </is>
       </c>
-      <c r="B51" s="9" t="inlineStr">
+      <c r="B51" s="10" t="inlineStr">
         <is>
           <t>ESP32-S3 devkit, 2.8" TFT, 45 mm faders, EC11s, buttons, LEDs, resistors</t>
         </is>
       </c>
-      <c r="C51" s="9" t="inlineStr">
+      <c r="C51" s="10" t="inlineStr">
         <is>
           <t>Already bought</t>
         </is>
       </c>
-      <c r="D51" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E51" s="10" t="n">
+      <c r="D51" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F51" s="10">
+      <c r="F51" s="11">
         <f>D51*E51</f>
         <v/>
       </c>
-      <c r="G51" s="9" t="inlineStr">
+      <c r="G51" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H51" s="9" t="inlineStr">
+      <c r="H51" s="10" t="inlineStr">
         <is>
           <t>owned</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="inlineStr">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>Controller</t>
         </is>
       </c>
-      <c r="B52" s="7" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>Headers</t>
         </is>
       </c>
-      <c r="C52" s="7" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>Female 2.54 mm strips</t>
         </is>
       </c>
-      <c r="D52" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E52" s="8" t="n">
+      <c r="D52" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F52" s="8">
+      <c r="F52" s="6">
         <f>D52*E52</f>
         <v/>
       </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="G52" s="5" t="inlineStr">
         <is>
           <t>AliExpress</t>
         </is>
       </c>
-      <c r="H52" s="7" t="inlineStr">
+      <c r="H52" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>Shipping</t>
         </is>
       </c>
-      <c r="B53" s="7" t="inlineStr">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>DigiKey / Mouser</t>
         </is>
       </c>
-      <c r="C53" s="7" t="inlineStr">
+      <c r="C53" s="5" t="inlineStr">
         <is>
           <t>Free over the order threshold</t>
         </is>
       </c>
-      <c r="D53" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E53" s="8" t="n">
+      <c r="D53" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F53" s="8">
+      <c r="F53" s="6">
         <f>D53*E53</f>
         <v/>
       </c>
-      <c r="G53" s="7" t="inlineStr">
+      <c r="G53" s="5" t="inlineStr">
         <is>
           <t>DigiKey</t>
         </is>
       </c>
-      <c r="H53" s="7" t="inlineStr">
+      <c r="H53" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="7" t="inlineStr">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>Shipping</t>
         </is>
       </c>
-      <c r="B54" s="7" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>Tayda</t>
         </is>
       </c>
-      <c r="C54" s="7" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>To US</t>
         </is>
       </c>
-      <c r="D54" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E54" s="8" t="n">
+      <c r="D54" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="F54" s="8">
+      <c r="F54" s="6">
         <f>D54*E54</f>
         <v/>
       </c>
-      <c r="G54" s="7" t="inlineStr">
+      <c r="G54" s="5" t="inlineStr">
         <is>
           <t>Tayda</t>
         </is>
       </c>
-      <c r="H54" s="7" t="inlineStr">
+      <c r="H54" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="inlineStr">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>Shipping</t>
         </is>
       </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>Jameco</t>
         </is>
       </c>
-      <c r="C55" s="7" t="inlineStr">
+      <c r="C55" s="5" t="inlineStr">
         <is>
           <t>Ground</t>
         </is>
       </c>
-      <c r="D55" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E55" s="8" t="n">
+      <c r="D55" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="F55" s="8">
+      <c r="F55" s="6">
         <f>D55*E55</f>
         <v/>
       </c>
-      <c r="G55" s="7" t="inlineStr">
+      <c r="G55" s="5" t="inlineStr">
         <is>
           <t>Jameco</t>
         </is>
       </c>
-      <c r="H55" s="7" t="inlineStr">
+      <c r="H55" s="5" t="inlineStr">
         <is>
           <t>estimate</t>
         </is>

</xml_diff>